<commit_message>
fix(classeurs): position des logos sur l'accueil, la méthodologie, la synthèse et la liste
Reprend les positions choisies à la main dans OnlyOffice. Le générateur
accepte une ancre par feuille (ANCRES_BANDEAU) ; un déplacement fait dans
une seule variante vaut pour les deux. Logo INR de « Liste ONR » placé
sous le tableau dans le modèle.

Signed-off-by: Guillaume G. <guillaume.gallon@gmail.com>
</commit_message>
<xml_diff>
--- a/INR_GPC_ONR Template.xlsx
+++ b/INR_GPC_ONR Template.xlsx
@@ -30268,10 +30268,10 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <xdr:oneCellAnchor>
     <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>114300</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>47625</xdr:rowOff>
+      <xdr:col>0</xdr:col>
+      <xdr:colOff>66674</xdr:colOff>
+      <xdr:row>32</xdr:row>
+      <xdr:rowOff>142874</xdr:rowOff>
     </xdr:from>
     <xdr:ext cx="2000250" cy="638175"/>
     <xdr:pic>

</xml_diff>